<commit_message>
docs: review-1 follow-ups (agents, kind rename, settings)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/source/Nexus_Phase1_Sprint_Plan.xlsx
+++ b/docs/source/Nexus_Phase1_Sprint_Plan.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint plan" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hiring" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Architecture" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Read me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sprint plan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Hiring" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Backlog" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Architecture" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Future" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Backlog'!$A$1:$O$76</definedName>
@@ -874,7 +874,7 @@
       </c>
       <c r="E4" s="19" t="inlineStr">
         <is>
-          <t>DATOMS API docs</t>
+          <t>DATOMS sample bulk response + bulk field list (Q21, Q22)</t>
         </is>
       </c>
       <c r="F4" s="19">
@@ -929,7 +929,7 @@
       </c>
       <c r="E5" s="19" t="inlineStr">
         <is>
-          <t>DATOMS API docs + key</t>
+          <t>DATOMS sample + field list (Q21, Q22) + key</t>
         </is>
       </c>
       <c r="F5" s="19">
@@ -984,7 +984,7 @@
       </c>
       <c r="E6" s="19" t="inlineStr">
         <is>
-          <t>Asset location + status in API</t>
+          <t>Bulk field names for location + status (Q22)</t>
         </is>
       </c>
       <c r="F6" s="19">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="E7" s="19" t="inlineStr">
         <is>
-          <t>Site totals in API</t>
+          <t>Whether DATOMS has site totals and ownership (Q3); field names (Q22)</t>
         </is>
       </c>
       <c r="F7" s="19">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="E8" s="19" t="inlineStr">
         <is>
-          <t>Notifications in API</t>
+          <t>Alert field names in the bulk response (Q22)</t>
         </is>
       </c>
       <c r="F8" s="19">
@@ -1381,6 +1381,7 @@
         <v/>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="15" customHeight="1" s="14">
       <c r="A15" s="22" t="inlineStr">
         <is>
@@ -2090,21 +2091,21 @@
       </c>
       <c r="E5" s="24" t="inlineStr">
         <is>
-          <t>Entra ID app registrations (API + web app), app roles, Nexus security groups</t>
+          <t>Entra ID app registrations (API + web app), Nexus security groups, app-assigned groups claim</t>
         </is>
       </c>
       <c r="F5" s="19" t="inlineStr">
         <is>
           <t>1. In Entra ID, register two apps: 'Nexus API' and 'Nexus Web'.
-2. On Nexus API, define app roles: Admin, Leadership, ProjectDirector, ProjectManager, HSE, Plant, Procurement.
-3. Create security groups (e.g. Nexus-Admins) and assign them to the roles.
+2. Create the Nexus security groups (docs/08 section 1; e.g. Nexus-Admins). Roles are mapped from groups in the Nexus database (docs/08 section 3), not defined as Entra app roles. The final role list is Q17.
+3. On Nexus API, set the groups claim to 'Groups assigned to the application' (ADR 0008). Assign the Nexus groups to the enterprise app; users must be direct members. No Graph permission or secret.
 4. Turn on 'assignment required' so only group members can sign in.
 5. Share client IDs with the frontend.</t>
         </is>
       </c>
       <c r="G5" s="19" t="inlineStr">
         <is>
-          <t>Sign-in apps and roles ready; test users in each group</t>
+          <t>Sign-in apps and groups ready; test users in each group</t>
         </is>
       </c>
       <c r="H5" s="19" t="inlineStr">
@@ -2125,7 +2126,7 @@
       <c r="K5" s="19" t="n"/>
       <c r="L5" s="19" t="inlineStr">
         <is>
-          <t>Entra admin consent</t>
+          <t>Entra admin consent; Entra ID P1 licence and setup confirmed by Innovo IT (Q16)</t>
         </is>
       </c>
       <c r="M5" s="19" t="n">
@@ -2138,7 +2139,7 @@
       </c>
       <c r="O5" s="19" t="inlineStr">
         <is>
-          <t>Test users in each group can get a token with the right role</t>
+          <t>Test users in each group get a token whose groups claim contains only their app-assigned Nexus group(s)</t>
         </is>
       </c>
     </row>
@@ -3183,16 +3184,16 @@
       </c>
       <c r="E20" s="24" t="inlineStr">
         <is>
-          <t>DATOMS API client: auth, paging, retries, rate-limit handling</t>
+          <t>DATOMS API client: bulk endpoint, paging, retries, rate-limit and credit handling</t>
         </is>
       </c>
       <c r="F20" s="19" t="inlineStr">
         <is>
-          <t>1. Read the DATOMS API docs (once received).
-2. Build a DATOMS client module: login/token, list sites, list devices, get values.
-3. Handle paging, retries and rate limits.
-4. Test against GHAFWOODS on dev.
-If docs are not here yet: build with a mock and swap later.</t>
+          <t>1. Read the v4 PDF, plus the DATOMS sample bulk response (Q21) and bulk field list (Q22) once received.
+2. Build packages/datoms-client: list assets (catalogue) and the bulk endpoint (fleet and id mode) as the ONLY telemetry source (ADR 0010). data/latest is for CLI checks only.
+3. Put ALL field mapping in src/mapping.ts. Until the sample arrives, build against the v4 PDF shape. Save the sample to fixtures/ with tokens removed.
+4. Handle paging, 422 halving (with the learned page size), retries, rate limits, and the credit budget with budget.max_share (ADR 0005).
+5. Test against GHAFWOODS on dev using fixtures or a small id-mode subset (never the full fleet from dev).</t>
         </is>
       </c>
       <c r="G20" s="19" t="inlineStr">
@@ -3218,7 +3219,7 @@
       <c r="K20" s="19" t="n"/>
       <c r="L20" s="19" t="inlineStr">
         <is>
-          <t>DATOMS API docs + read-only key</t>
+          <t>DATOMS sample bulk response (Q21) + bulk field list (Q22) + read-only key. Needed before this task starts; they do not block S0 or S1.</t>
         </is>
       </c>
       <c r="M20" s="19" t="n">
@@ -3231,7 +3232,7 @@
       </c>
       <c r="O20" s="19" t="inlineStr">
         <is>
-          <t>Client reads GHAFWOODS sites and devices in dev</t>
+          <t>Client reads the GHAFWOODS demo fleet (generators and tower cranes) through the bulk endpoint in dev; DATOMS field names exist only in src/mapping.ts</t>
         </is>
       </c>
     </row>
@@ -3557,9 +3558,10 @@
       </c>
       <c r="F25" s="19" t="inlineStr">
         <is>
-          <t>1. Scheduled job in apps/worker, every hour.
-2. Read all DATOMS sites, devices and parameters (name, unit).
-3. Insert new ones, update changed ones in the database.</t>
+          <t>1. Scheduled job in apps/worker, every hour (and early when the poll sees unknown ids).
+2. Read all DATOMS assets (list assets: names, nameplate). Sites, asset types and parameters (name, unit) come in the bulk rows. The live poll (S3-03) upserts them the same way, so the catalogue job spends no bulk credits.
+3. Insert new ones, update changed ones in the database.
+4. Retire safely (docs/07 section 6): only after a complete walk; only rows missed in 2 consecutive complete walks; retire nothing and alert if more than 5% would go.</t>
         </is>
       </c>
       <c r="G25" s="19" t="inlineStr">
@@ -3589,7 +3591,7 @@
       </c>
       <c r="L25" s="19" t="inlineStr">
         <is>
-          <t>DATOMS API docs + read-only key</t>
+          <t>DATOMS sample + field list (Q21, Q22) + read-only key; id stability (Q11)</t>
         </is>
       </c>
       <c r="M25" s="19" t="n">
@@ -3702,20 +3704,20 @@
       </c>
       <c r="E27" s="24" t="inlineStr">
         <is>
-          <t>Live sync (every minute): latest values and statuses to readings + latest value table</t>
+          <t>Live sync (every minute by default): bulk endpoint → packets, latest values, statuses, locations, alerts</t>
         </is>
       </c>
       <c r="F27" s="19" t="inlineStr">
         <is>
-          <t>1. Job every minute: get latest values and statuses for all devices.
-2. Write them to 'reading' (history) and 'latest_value' (current).
-3. Insert in batches.
-4. Log how long each run takes.</t>
+          <t>1. Job every 60 s by default (per-type interval, ADR 0006): bulk endpoint only (ADR 0010). Fleet mode when every asset is due, otherwise id mode. In dev, only the configured subset (ADR 0005).
+2. Write telemetry.packet (history) and telemetry.latest_packet (current); status, location and alerts on change only.
+3. Insert in batches. No per-poll bookkeeping writes (asset_parameter is insert-only; status observed_at only on change).
+4. Log how long each run takes and the credits used per window.</t>
         </is>
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>Live DATOMS data in Nexus within 60 seconds</t>
+          <t>Live DATOMS data in Nexus within about 2 poll intervals</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
@@ -3749,7 +3751,7 @@
       </c>
       <c r="O27" s="19" t="inlineStr">
         <is>
-          <t>Value in Nexus within 60 s of DATOMS</t>
+          <t>Value in Nexus within 2 poll intervals of DATOMS (N-03)</t>
         </is>
       </c>
     </row>
@@ -3776,7 +3778,7 @@
       </c>
       <c r="E28" s="24" t="inlineStr">
         <is>
-          <t>History backfill and gap repair after outages</t>
+          <t>History backfill and gap repair after outages (ON HOLD)</t>
         </is>
       </c>
       <c r="F28" s="19" t="inlineStr">
@@ -3812,13 +3814,17 @@
           <t>S3-03</t>
         </is>
       </c>
-      <c r="L28" s="19" t="n"/>
+      <c r="L28" s="19" t="inlineStr">
+        <is>
+          <t>ON HOLD (decided 2026-10-08). The bulk endpoint has no history (ADR 0010); Nexus builds its own history from polls from day one. Needs a DATOMS history feed (Q12) and a new ADR to use it. Until then, gaps stay gaps and charts show coverage (ADR 0007).</t>
+        </is>
+      </c>
       <c r="M28" s="19" t="n">
         <v>2</v>
       </c>
       <c r="N28" s="25" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="O28" s="19" t="inlineStr">
@@ -4073,8 +4079,9 @@
       <c r="F32" s="19" t="inlineStr">
         <is>
           <t>1. Use the rollup functions in db/schema.sql: telemetry.refresh_rollup_5m and refresh_rollup_combine (1 h, 1 day in Asia/Dubai).
-2. Worker rollups job runs every minute for the recent window and re-runs for late data.
-3. Check a 30-day query returns in under 1 second.</t>
+2. Worker rollups job (ADR 0007): refresh_rollup_5m once per CLOSED 5-minute bucket, 2 poll intervals after it ends; re-run only for closed buckets that get late packets; 1 h after the hour's last bucket; 1 d after the Dubai day. No sliding window, no in-memory accumulators.
+3. Return data coverage (packets / expectedPackets) with each bucket.
+4. Check a 30-day query returns in under 1 second.</t>
         </is>
       </c>
       <c r="G32" s="19" t="inlineStr">
@@ -4145,8 +4152,9 @@
       </c>
       <c r="F33" s="19" t="inlineStr">
         <is>
-          <t>1. When the worker sees a status or value change, publish a message to Azure Web PubSub (per project channel).
-2. API gives the browser a Web PubSub token for only the projects it may see.</t>
+          <t>1. When the worker sees a status or location change, publish a slim message to Azure Web PubSub (per project group): no parameter values; values.updated hint; summary.updated; chunked well under 1 MB (docs/10, ADR 0008).
+2. API gives the browser a Web PubSub token with no group-join rights. POST /v1/live/subscriptions checks permission and scope, then joins the connection to project groups on the server.
+3. On any Nexus access change, close the affected live connections so clients re-subscribe through the scope check. Settle with the security-reviewer how the API confirms a connectionId belongs to the caller.</t>
         </is>
       </c>
       <c r="G33" s="19" t="inlineStr">
@@ -4185,7 +4193,7 @@
       </c>
       <c r="O33" s="19" t="inlineStr">
         <is>
-          <t>Pin colour changes without refresh</t>
+          <t>Pin colour changes without refresh; a user whose project access is removed stops receiving that project's messages at once; nothing project-specific is sent to the portfolio group</t>
         </is>
       </c>
     </row>
@@ -4212,18 +4220,18 @@
       </c>
       <c r="E34" s="24" t="inlineStr">
         <is>
-          <t>Project summary API for the equipment and energy info boxes</t>
+          <t>Project summary APIs for the equipment and energy info boxes</t>
         </is>
       </c>
       <c r="F34" s="19" t="inlineStr">
         <is>
-          <t>1. Endpoint GET /projects/{id}/summary returning the equipment and energy info boxes.
-2. Fill them from latest DATOMS values. Manpower and materials are added later once their source is known.</t>
+          <t>1. Endpoints GET /projects/{id}/equipment/summary (Box 2) and GET /projects/{id}/energy/summary (Box 3), as in docs/10.
+2. Fill them from the latest DATOMS values: equipment counts from kind = 'physical' assets; energy site totals from site_metric records when DATOMS provides them. Manpower and materials are not built (slots only).</t>
         </is>
       </c>
       <c r="G34" s="19" t="inlineStr">
         <is>
-          <t>One call loads the project page</t>
+          <t>The project page loads its boxes</t>
         </is>
       </c>
       <c r="H34" s="19" t="inlineStr">
@@ -4257,7 +4265,7 @@
       </c>
       <c r="O34" s="19" t="inlineStr">
         <is>
-          <t>One call returns all four boxes</t>
+          <t>The two endpoints return Box 2 and Box 3 as reported; Boxes 1 and 4 are "coming later" slots</t>
         </is>
       </c>
     </row>
@@ -4362,10 +4370,10 @@
       </c>
       <c r="F36" s="19" t="inlineStr">
         <is>
-          <t>1. Draw one pin per asset at its DATOMS location.
-2. Icon by type: tower crane, hoist, equipment, generator.
+          <t>1. Draw one pin per equipment asset (kind = 'physical') at its DATOMS location; no location = "Not on map".
+2. Icon by type: tower crane, hoist, equipment, generator; unknown types use the generic icon.
 3. Colour by DATOMS status: Running green, Idle amber, Maintenance red, Off grey.
-4. Turn on clustering and a Map/Satellite switch.</t>
+4. Turn on clustering and a Map/Satellite switch. 3D uses the same icons with no callouts or pulse (ADR 0008).</t>
         </is>
       </c>
       <c r="G36" s="19" t="inlineStr">
@@ -4395,7 +4403,7 @@
       </c>
       <c r="L36" s="19" t="inlineStr">
         <is>
-          <t>DATOMS: does API return location + status?</t>
+          <t>Bulk field names for location + status (Q22; DATOMS confirmed the data is in the bulk response); blink vs pulse (Q19)</t>
         </is>
       </c>
       <c r="M36" s="19" t="n">
@@ -4584,7 +4592,7 @@
       </c>
       <c r="F39" s="19" t="inlineStr">
         <is>
-          <t>1. Endpoint returning per project: generators (running/total), solar generation, mains, total load, loads by area, site totals and CO2 exactly as DATOMS gives them.
+          <t>1. Endpoint returning per project: generators (running/total), solar generation, mains, total load, loads by area, site totals and CO2 exactly as DATOMS gives them in the bulk response. Site totals are read from site_metric records (ADR 0009); anything missing shows "no data yet".
 2. Compare with the DATOMS Site View for GHAFWOODS; numbers must match.</t>
         </is>
       </c>
@@ -4615,7 +4623,7 @@
       </c>
       <c r="L39" s="19" t="inlineStr">
         <is>
-          <t>DATOMS: are site totals in the API?</t>
+          <t>Whether DATOMS has site totals (Q3); bulk field names (Q22)</t>
         </is>
       </c>
       <c r="M39" s="19" t="n">
@@ -4661,7 +4669,7 @@
       <c r="F40" s="19" t="inlineStr">
         <is>
           <t>1. Endpoint listing energy equipment: DG ID, description, type (DG/solar/mains), status, owned or hired.
-2. Ownership comes from the Nexus asset register.</t>
+2. Ownership comes from a DATOMS field (R-31). If DATOMS lacks it, the column is hidden and reported (Q3). Nexus doesn't keep its own ownership register.</t>
         </is>
       </c>
       <c r="G40" s="19" t="inlineStr">
@@ -4733,7 +4741,7 @@
       <c r="F41" s="19" t="inlineStr">
         <is>
           <t>1. Endpoints for trends by day, week, month, year.
-2. Read from the summaries in S5-01, never raw readings.</t>
+2. Read from the rollup tables (S4-01), never raw readings for ranges over 6 h. 5-minute data only within 60 days; older ranges use hourly. Return the resolution used and data coverage per bucket.</t>
         </is>
       </c>
       <c r="G41" s="19" t="inlineStr">
@@ -5161,8 +5169,8 @@
       </c>
       <c r="F47" s="19" t="inlineStr">
         <is>
-          <t>1. Endpoint listing equipment per project: ID, name, type, make/model, current status.
-2. Include every extra parameter DATOMS sends for that device.</t>
+          <t>1. Endpoint listing equipment per project (kind = 'physical' only): ID, name, type, make/model, current status, plus extra nameplate fields as optional columns.
+2. Every parameter DATOMS sends for a device is available from GET /assets/{id} (device card). The list endpoint carries no live values (ADR 0008).</t>
         </is>
       </c>
       <c r="G47" s="19" t="inlineStr">
@@ -5234,7 +5242,7 @@
       <c r="F48" s="19" t="inlineStr">
         <is>
           <t>1. Endpoint for one device: latest values of every parameter.
-2. Today's timeline of status changes (running, idle, off) from DATOMS events.</t>
+2. Today's timeline of status changes (running, idle, off) as observed by Nexus in polls, labelled "observed by Nexus" (ADR 0007). DATOMS's own status history is used only if a later ADR adds it.</t>
         </is>
       </c>
       <c r="G48" s="19" t="inlineStr">
@@ -5273,7 +5281,7 @@
       </c>
       <c r="O48" s="19" t="inlineStr">
         <is>
-          <t>Timeline matches DATOMS events</t>
+          <t>Timeline shows the status changes Nexus observed, labelled "observed by Nexus", accurate to one poll interval</t>
         </is>
       </c>
     </row>
@@ -5305,7 +5313,7 @@
       </c>
       <c r="F49" s="19" t="inlineStr">
         <is>
-          <t>1. Counts per project: tower cranes total/idle, hoists total/idle, all equipment total/idle, using DATOMS statuses.
+          <t>1. Counts per project (kind = 'physical' only): tower cranes total/idle, hoists total/idle, all equipment total/idle, using DATOMS statuses.
 2. Add to the project summary (S5-03).</t>
         </is>
       </c>
@@ -5372,13 +5380,13 @@
       </c>
       <c r="E50" s="24" t="inlineStr">
         <is>
-          <t>Notifications sync from DATOMS and API (filter by site, asset, type)</t>
+          <t>Notifications from the DATOMS bulk response, and API (filter by site, asset, type)</t>
         </is>
       </c>
       <c r="F50" s="19" t="inlineStr">
         <is>
-          <t>1. Worker job every minute: fetch DATOMS notifications and faults.
-2. Store them; endpoint to list with filters: site, asset, type, date.
+          <t>1. In the live poll: take DATOMS alerts and faults from the bulk response (ADR 0010; no separate events job).
+2. Store them; endpoint to list with filters: site, asset, type, date. "Mark all read" moves a read marker (docs/06 section 3, item 11).
 3. Show them exactly as DATOMS sends them.</t>
         </is>
       </c>
@@ -5404,12 +5412,12 @@
       </c>
       <c r="K50" s="19" t="inlineStr">
         <is>
-          <t>S3-01</t>
+          <t>S3-03</t>
         </is>
       </c>
       <c r="L50" s="19" t="inlineStr">
         <is>
-          <t>DATOMS: notifications in API?</t>
+          <t>Alert field names in the bulk response (Q22)</t>
         </is>
       </c>
       <c r="M50" s="19" t="n">
@@ -6728,7 +6736,7 @@
       </c>
       <c r="F69" s="19" t="inlineStr">
         <is>
-          <t>1. Give pilot users access on GHAFWOODS.
+          <t>1. Give pilot users access on GHAFWOODS in **prod** (there is no test environment, ADR 0008): only pilot users are assigned to the Entra app during the pilot.
 2. Walk through each screen with them.
 3. Record issues in the backlog.</t>
         </is>
@@ -7246,6 +7254,7 @@
         </is>
       </c>
     </row>
+    <row r="77"/>
     <row r="78" ht="15" customHeight="1" s="14">
       <c r="L78" s="16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore: tidy settings and architecture sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/source/Nexus_Phase1_Sprint_Plan.xlsx
+++ b/docs/source/Nexus_Phase1_Sprint_Plan.xlsx
@@ -1381,7 +1381,6 @@
         <v/>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="15" customHeight="1" s="14">
       <c r="A15" s="22" t="inlineStr">
         <is>
@@ -7254,7 +7253,6 @@
         </is>
       </c>
     </row>
-    <row r="77"/>
     <row r="78" ht="15" customHeight="1" s="14">
       <c r="L78" s="16" t="inlineStr">
         <is>
@@ -7427,7 +7425,7 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>Same codebase, separate process: catalogue hourly, live values and notifications every minute, history backfill, gap repair</t>
+          <t>Same codebase, separate process: catalogue hourly, live values and notifications every minute (history backfill on hold, see S3-04)</t>
         </is>
       </c>
       <c r="C8" s="19" t="inlineStr">

</xml_diff>

<commit_message>
docs: S7-02 CSP step in sprint sheet
- Nexus_Phase1_Sprint_Plan.xlsx (Backlog, row 56): S7-02 gets step 4 (web
  CSP and security headers, docs/08 s6), plus the matching task title,
  output and acceptance check; row height raised to fit. Formulas,
  the Status dropdown, conditional formatting and styles are unchanged.
- backlog.md regenerated from the sheet. Against main the only change is
  the S7-02 block; step 4 is now plain text, matching the sheet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/source/Nexus_Phase1_Sprint_Plan.xlsx
+++ b/docs/source/Nexus_Phase1_Sprint_Plan.xlsx
@@ -5794,7 +5794,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="35.05" customHeight="1" s="14">
+    <row r="56" ht="79.84999999999999" customHeight="1" s="14">
       <c r="A56" s="19" t="inlineStr">
         <is>
           <t>S7-02</t>
@@ -5817,19 +5817,20 @@
       </c>
       <c r="E56" s="24" t="inlineStr">
         <is>
-          <t>Security hardening: private endpoints, key rotation, firewall rules</t>
+          <t>Security hardening: private endpoints, key rotation, firewall rules, web security headers</t>
         </is>
       </c>
       <c r="F56" s="19" t="inlineStr">
         <is>
           <t>1. Put PostgreSQL and Blob behind private endpoints.
 2. Rotate keys in Key Vault.
-3. Firewall: only Container Apps can reach the database.</t>
+3. Firewall: only Container Apps can reach the database.
+4. Web app security headers and CSP (docs/08 §6) in staticwebapp.config.json: a CSP that allows only the MSAL (Entra) and ArcGIS domains plus the API and Web PubSub hosts; HSTS, X-Content-Type-Options, Referrer-Policy, frame-ancestors none. (Added by the S0 plan, 2026-10-09.)</t>
         </is>
       </c>
       <c r="G56" s="19" t="inlineStr">
         <is>
-          <t>Data not reachable from the internet</t>
+          <t>Data not reachable from the internet; the web app sends a CSP and security headers</t>
         </is>
       </c>
       <c r="H56" s="19" t="inlineStr">
@@ -5859,7 +5860,7 @@
       </c>
       <c r="O56" s="19" t="inlineStr">
         <is>
-          <t>Databases unreachable from internet</t>
+          <t>Databases unreachable from internet; a header scan of the prod web URL shows the CSP and security headers, and sign-in and the map still work with the CSP on</t>
         </is>
       </c>
     </row>

</xml_diff>